<commit_message>
Fixes format of the data for TP time progressions and added omnium GRAPH
</commit_message>
<xml_diff>
--- a/pages/WR_progressions/Mens_Progression.xlsx
+++ b/pages/WR_progressions/Mens_Progression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sportnzgroup-my.sharepoint.com/personal/anja_kuys_hpsnz_org_nz/Documents/Desktop/Scripts/CNZPD/pages/WR_progressions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_FF6BE833DD9E4E317729F09F5470CA66DBC2C15B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{58490DAC-1E65-4B53-9254-F8071515AB94}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="11_FF6BE833DD9E4E317729F09F5470CA66DBC2C15B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{610C50C8-F9F7-47E4-AF08-BD29EACE8B55}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Medals_F200" sheetId="1" r:id="rId1"/>
@@ -20289,7 +20289,6 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:L133"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -20345,7 +20344,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="2" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="23" t="s">
         <v>25</v>
       </c>
@@ -20383,7 +20382,7 @@
         <v>56.962000000000003</v>
       </c>
     </row>
-    <row r="3" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="23" t="s">
         <v>25</v>
       </c>
@@ -20421,7 +20420,7 @@
         <v>56.962000000000003</v>
       </c>
     </row>
-    <row r="4" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="23" t="s">
         <v>25</v>
       </c>
@@ -20459,7 +20458,7 @@
         <v>56.962000000000003</v>
       </c>
     </row>
-    <row r="5" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" s="25" t="s">
         <v>27</v>
       </c>
@@ -20497,7 +20496,7 @@
         <v>61.537999999999997</v>
       </c>
     </row>
-    <row r="6" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" s="25" t="s">
         <v>27</v>
       </c>
@@ -20535,7 +20534,7 @@
         <v>61.537999999999997</v>
       </c>
     </row>
-    <row r="7" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" s="25" t="s">
         <v>27</v>
       </c>
@@ -20687,7 +20686,7 @@
         <v>57.6</v>
       </c>
     </row>
-    <row r="11" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11" s="25" t="s">
         <v>30</v>
       </c>
@@ -20725,7 +20724,7 @@
         <v>58.536585365853668</v>
       </c>
     </row>
-    <row r="12" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" s="25" t="s">
         <v>30</v>
       </c>
@@ -20763,7 +20762,7 @@
         <v>58.536585365853668</v>
       </c>
     </row>
-    <row r="13" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13" s="25" t="s">
         <v>30</v>
       </c>
@@ -20915,7 +20914,7 @@
         <v>58.158000000000001</v>
       </c>
     </row>
-    <row r="17" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A17" s="25" t="s">
         <v>32</v>
       </c>
@@ -20953,7 +20952,7 @@
         <v>55.988</v>
       </c>
     </row>
-    <row r="18" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A18" s="25" t="s">
         <v>32</v>
       </c>
@@ -20991,7 +20990,7 @@
         <v>55.988</v>
       </c>
     </row>
-    <row r="19" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A19" s="25" t="s">
         <v>32</v>
       </c>
@@ -21029,7 +21028,7 @@
         <v>55.988</v>
       </c>
     </row>
-    <row r="20" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A20" s="23" t="s">
         <v>34</v>
       </c>
@@ -21067,7 +21066,7 @@
         <v>52.786000000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A21" s="23" t="s">
         <v>34</v>
       </c>
@@ -21105,7 +21104,7 @@
         <v>52.786000000000001</v>
       </c>
     </row>
-    <row r="22" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A22" s="23" t="s">
         <v>34</v>
       </c>
@@ -21143,7 +21142,7 @@
         <v>52.786000000000001</v>
       </c>
     </row>
-    <row r="23" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A23" s="25" t="s">
         <v>27</v>
       </c>
@@ -21181,7 +21180,7 @@
         <v>57.6</v>
       </c>
     </row>
-    <row r="24" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A24" s="25" t="s">
         <v>27</v>
       </c>
@@ -21219,7 +21218,7 @@
         <v>57.6</v>
       </c>
     </row>
-    <row r="25" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A25" s="25" t="s">
         <v>27</v>
       </c>
@@ -21257,7 +21256,7 @@
         <v>57.6</v>
       </c>
     </row>
-    <row r="26" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A26" s="23" t="s">
         <v>35</v>
       </c>
@@ -21295,7 +21294,7 @@
         <v>53.811999999999998</v>
       </c>
     </row>
-    <row r="27" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A27" s="23" t="s">
         <v>35</v>
       </c>
@@ -21333,7 +21332,7 @@
         <v>53.811999999999998</v>
       </c>
     </row>
-    <row r="28" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A28" s="23" t="s">
         <v>35</v>
       </c>
@@ -21485,7 +21484,7 @@
         <v>56.515000000000001</v>
       </c>
     </row>
-    <row r="32" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A32" s="23" t="s">
         <v>34</v>
       </c>
@@ -21523,7 +21522,7 @@
         <v>57.234000000000002</v>
       </c>
     </row>
-    <row r="33" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A33" s="23" t="s">
         <v>34</v>
       </c>
@@ -21561,7 +21560,7 @@
         <v>57.234000000000002</v>
       </c>
     </row>
-    <row r="34" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A34" s="23" t="s">
         <v>34</v>
       </c>
@@ -21599,7 +21598,7 @@
         <v>57.234000000000002</v>
       </c>
     </row>
-    <row r="35" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A35" s="25" t="s">
         <v>37</v>
       </c>
@@ -21637,7 +21636,7 @@
         <v>53.651000000000003</v>
       </c>
     </row>
-    <row r="36" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A36" s="25" t="s">
         <v>37</v>
       </c>
@@ -21675,7 +21674,7 @@
         <v>53.651000000000003</v>
       </c>
     </row>
-    <row r="37" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A37" s="25" t="s">
         <v>37</v>
       </c>
@@ -21713,7 +21712,7 @@
         <v>53.651000000000003</v>
       </c>
     </row>
-    <row r="38" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A38" s="23" t="s">
         <v>38</v>
       </c>
@@ -21751,7 +21750,7 @@
         <v>38.256999999999998</v>
       </c>
     </row>
-    <row r="39" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A39" s="23" t="s">
         <v>38</v>
       </c>
@@ -21789,7 +21788,7 @@
         <v>38.256999999999998</v>
       </c>
     </row>
-    <row r="40" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A40" s="23" t="s">
         <v>38</v>
       </c>
@@ -21935,7 +21934,7 @@
       </c>
       <c r="L43" s="25"/>
     </row>
-    <row r="44" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A44" s="23" t="s">
         <v>39</v>
       </c>
@@ -21973,7 +21972,7 @@
         <v>52.709000000000003</v>
       </c>
     </row>
-    <row r="45" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A45" s="23" t="s">
         <v>39</v>
       </c>
@@ -22011,7 +22010,7 @@
         <v>52.709000000000003</v>
       </c>
     </row>
-    <row r="46" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A46" s="23" t="s">
         <v>39</v>
       </c>
@@ -22049,7 +22048,7 @@
         <v>52.709000000000003</v>
       </c>
     </row>
-    <row r="47" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A47" s="25" t="s">
         <v>34</v>
       </c>
@@ -22087,7 +22086,7 @@
         <v>57.784999999999997</v>
       </c>
     </row>
-    <row r="48" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A48" s="25" t="s">
         <v>34</v>
       </c>
@@ -22125,7 +22124,7 @@
         <v>57.784999999999997</v>
       </c>
     </row>
-    <row r="49" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A49" s="25" t="s">
         <v>34</v>
       </c>
@@ -22163,7 +22162,7 @@
         <v>57.784999999999997</v>
       </c>
     </row>
-    <row r="50" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A50" s="23" t="s">
         <v>36</v>
       </c>
@@ -22201,7 +22200,7 @@
         <v>56.161999999999999</v>
       </c>
     </row>
-    <row r="51" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A51" s="23" t="s">
         <v>36</v>
       </c>
@@ -22239,7 +22238,7 @@
         <v>56.161999999999999</v>
       </c>
     </row>
-    <row r="52" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A52" s="23" t="s">
         <v>36</v>
       </c>
@@ -22391,7 +22390,7 @@
         <v>57.052</v>
       </c>
     </row>
-    <row r="56" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A56" s="23" t="s">
         <v>39</v>
       </c>
@@ -22429,7 +22428,7 @@
         <v>53.695999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A57" s="23" t="s">
         <v>39</v>
       </c>
@@ -22467,7 +22466,7 @@
         <v>53.695999999999998</v>
       </c>
     </row>
-    <row r="58" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A58" s="23" t="s">
         <v>39</v>
       </c>
@@ -22505,7 +22504,7 @@
         <v>53.695999999999998</v>
       </c>
     </row>
-    <row r="59" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A59" s="25" t="s">
         <v>41</v>
       </c>
@@ -22543,7 +22542,7 @@
         <v>56.927999999999997</v>
       </c>
     </row>
-    <row r="60" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A60" s="25" t="s">
         <v>41</v>
       </c>
@@ -22581,7 +22580,7 @@
         <v>56.927999999999997</v>
       </c>
     </row>
-    <row r="61" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A61" s="25" t="s">
         <v>41</v>
       </c>
@@ -22619,7 +22618,7 @@
         <v>56.927999999999997</v>
       </c>
     </row>
-    <row r="62" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A62" s="23" t="s">
         <v>42</v>
       </c>
@@ -22657,7 +22656,7 @@
         <v>54.893999999999998</v>
       </c>
     </row>
-    <row r="63" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A63" s="23" t="s">
         <v>42</v>
       </c>
@@ -22695,7 +22694,7 @@
         <v>54.893999999999998</v>
       </c>
     </row>
-    <row r="64" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A64" s="23" t="s">
         <v>42</v>
       </c>
@@ -22847,7 +22846,7 @@
         <v>57.43</v>
       </c>
     </row>
-    <row r="68" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A68" s="23" t="s">
         <v>34</v>
       </c>
@@ -22885,7 +22884,7 @@
         <v>53.741</v>
       </c>
     </row>
-    <row r="69" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A69" s="23" t="s">
         <v>34</v>
       </c>
@@ -22923,7 +22922,7 @@
         <v>53.741</v>
       </c>
     </row>
-    <row r="70" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A70" s="23" t="s">
         <v>34</v>
       </c>
@@ -22961,7 +22960,7 @@
         <v>53.741</v>
       </c>
     </row>
-    <row r="71" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A71" s="25" t="s">
         <v>44</v>
       </c>
@@ -22999,7 +22998,7 @@
         <v>54.131999999999998</v>
       </c>
     </row>
-    <row r="72" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A72" s="25" t="s">
         <v>44</v>
       </c>
@@ -23037,7 +23036,7 @@
         <v>54.131999999999998</v>
       </c>
     </row>
-    <row r="73" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A73" s="25" t="s">
         <v>44</v>
       </c>
@@ -23075,7 +23074,7 @@
         <v>54.131999999999998</v>
       </c>
     </row>
-    <row r="74" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A74" s="23" t="s">
         <v>45</v>
       </c>
@@ -23113,7 +23112,7 @@
         <v>55.6</v>
       </c>
     </row>
-    <row r="75" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A75" s="23" t="s">
         <v>45</v>
       </c>
@@ -23151,7 +23150,7 @@
         <v>55.6</v>
       </c>
     </row>
-    <row r="76" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A76" s="23" t="s">
         <v>45</v>
       </c>
@@ -23189,7 +23188,7 @@
         <v>55.6</v>
       </c>
     </row>
-    <row r="77" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A77" s="25" t="s">
         <v>27</v>
       </c>
@@ -23227,7 +23226,7 @@
         <v>56.533000000000001</v>
       </c>
     </row>
-    <row r="78" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A78" s="25" t="s">
         <v>27</v>
       </c>
@@ -23265,7 +23264,7 @@
         <v>56.533000000000001</v>
       </c>
     </row>
-    <row r="79" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A79" s="25" t="s">
         <v>27</v>
       </c>
@@ -23303,7 +23302,7 @@
         <v>56.533000000000001</v>
       </c>
     </row>
-    <row r="80" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A80" s="23" t="s">
         <v>36</v>
       </c>
@@ -23341,7 +23340,7 @@
         <v>56.436</v>
       </c>
     </row>
-    <row r="81" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A81" s="23" t="s">
         <v>36</v>
       </c>
@@ -23379,7 +23378,7 @@
         <v>56.436</v>
       </c>
     </row>
-    <row r="82" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A82" s="23" t="s">
         <v>36</v>
       </c>
@@ -23417,7 +23416,7 @@
         <v>56.436</v>
       </c>
     </row>
-    <row r="83" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A83" s="25" t="s">
         <v>46</v>
       </c>
@@ -23455,7 +23454,7 @@
         <v>56.390999999999998</v>
       </c>
     </row>
-    <row r="84" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A84" s="25" t="s">
         <v>46</v>
       </c>
@@ -23493,7 +23492,7 @@
         <v>56.390999999999998</v>
       </c>
     </row>
-    <row r="85" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A85" s="25" t="s">
         <v>46</v>
       </c>
@@ -23645,7 +23644,7 @@
         <v>56.91</v>
       </c>
     </row>
-    <row r="89" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A89" s="25" t="s">
         <v>27</v>
       </c>
@@ -23683,7 +23682,7 @@
         <v>58.8</v>
       </c>
     </row>
-    <row r="90" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A90" s="25" t="s">
         <v>27</v>
       </c>
@@ -23721,7 +23720,7 @@
         <v>58.8</v>
       </c>
     </row>
-    <row r="91" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A91" s="25" t="s">
         <v>27</v>
       </c>
@@ -23759,7 +23758,7 @@
         <v>58.8</v>
       </c>
     </row>
-    <row r="92" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A92" s="23" t="s">
         <v>45</v>
       </c>
@@ -23797,7 +23796,7 @@
         <v>55.996000000000002</v>
       </c>
     </row>
-    <row r="93" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A93" s="23" t="s">
         <v>45</v>
       </c>
@@ -23835,7 +23834,7 @@
         <v>55.996000000000002</v>
       </c>
     </row>
-    <row r="94" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A94" s="23" t="s">
         <v>45</v>
       </c>
@@ -23873,7 +23872,7 @@
         <v>55.996000000000002</v>
       </c>
     </row>
-    <row r="95" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A95" s="25" t="s">
         <v>49</v>
       </c>
@@ -23911,7 +23910,7 @@
         <v>56.902000000000001</v>
       </c>
     </row>
-    <row r="96" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A96" s="25" t="s">
         <v>49</v>
       </c>
@@ -23949,7 +23948,7 @@
         <v>56.902000000000001</v>
       </c>
     </row>
-    <row r="97" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A97" s="25" t="s">
         <v>49</v>
       </c>
@@ -23987,7 +23986,7 @@
         <v>56.902000000000001</v>
       </c>
     </row>
-    <row r="98" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A98" s="23" t="s">
         <v>43</v>
       </c>
@@ -24025,7 +24024,7 @@
         <v>55.228000000000002</v>
       </c>
     </row>
-    <row r="99" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A99" s="23" t="s">
         <v>43</v>
       </c>
@@ -24063,7 +24062,7 @@
         <v>55.228000000000002</v>
       </c>
     </row>
-    <row r="100" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A100" s="23" t="s">
         <v>43</v>
       </c>
@@ -24101,7 +24100,7 @@
         <v>55.228000000000002</v>
       </c>
     </row>
-    <row r="101" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A101" s="25" t="s">
         <v>34</v>
       </c>
@@ -24137,7 +24136,7 @@
         <v>56.639000000000003</v>
       </c>
     </row>
-    <row r="102" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A102" s="25" t="s">
         <v>34</v>
       </c>
@@ -24173,7 +24172,7 @@
         <v>56.639000000000003</v>
       </c>
     </row>
-    <row r="103" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A103" s="25" t="s">
         <v>34</v>
       </c>
@@ -24209,7 +24208,7 @@
         <v>56.639000000000003</v>
       </c>
     </row>
-    <row r="104" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A104" s="23" t="s">
         <v>32</v>
       </c>
@@ -24245,7 +24244,7 @@
         <v>54.497999999999998</v>
       </c>
     </row>
-    <row r="105" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A105" s="23" t="s">
         <v>32</v>
       </c>
@@ -24281,7 +24280,7 @@
         <v>54.497999999999998</v>
       </c>
     </row>
-    <row r="106" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A106" s="23" t="s">
         <v>32</v>
       </c>
@@ -24317,7 +24316,7 @@
         <v>54.497999999999998</v>
       </c>
     </row>
-    <row r="107" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A107" s="25" t="s">
         <v>48</v>
       </c>
@@ -24328,7 +24327,7 @@
         <v>43162</v>
       </c>
       <c r="D107" s="25" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E107" s="25" t="s">
         <v>222</v>
@@ -24353,7 +24352,7 @@
         <v>43.445999999999998</v>
       </c>
     </row>
-    <row r="108" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A108" s="25" t="s">
         <v>48</v>
       </c>
@@ -24364,7 +24363,7 @@
         <v>43162</v>
       </c>
       <c r="D108" s="25" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E108" s="25" t="s">
         <v>223</v>
@@ -24389,7 +24388,7 @@
         <v>43.445999999999998</v>
       </c>
     </row>
-    <row r="109" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A109" s="25" t="s">
         <v>48</v>
       </c>
@@ -24400,7 +24399,7 @@
         <v>43162</v>
       </c>
       <c r="D109" s="25" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E109" s="25" t="s">
         <v>120</v>
@@ -24425,7 +24424,7 @@
         <v>43.445999999999998</v>
       </c>
     </row>
-    <row r="110" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A110" s="23" t="s">
         <v>46</v>
       </c>
@@ -24461,7 +24460,7 @@
         <v>53.319000000000003</v>
       </c>
     </row>
-    <row r="111" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A111" s="23" t="s">
         <v>46</v>
       </c>
@@ -24497,7 +24496,7 @@
         <v>53.319000000000003</v>
       </c>
     </row>
-    <row r="112" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A112" s="23" t="s">
         <v>46</v>
       </c>
@@ -24533,7 +24532,7 @@
         <v>53.319000000000003</v>
       </c>
     </row>
-    <row r="113" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A113" s="25" t="s">
         <v>28</v>
       </c>
@@ -24569,7 +24568,7 @@
         <v>52.246000000000002</v>
       </c>
     </row>
-    <row r="114" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A114" s="25" t="s">
         <v>28</v>
       </c>
@@ -24605,7 +24604,7 @@
         <v>52.246000000000002</v>
       </c>
     </row>
-    <row r="115" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A115" s="25" t="s">
         <v>28</v>
       </c>
@@ -24641,7 +24640,7 @@
         <v>52.246000000000002</v>
       </c>
     </row>
-    <row r="116" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A116" s="23" t="s">
         <v>34</v>
       </c>
@@ -24677,7 +24676,7 @@
         <v>54.948</v>
       </c>
     </row>
-    <row r="117" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A117" s="23" t="s">
         <v>34</v>
       </c>
@@ -24713,7 +24712,7 @@
         <v>54.948</v>
       </c>
     </row>
-    <row r="118" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A118" s="23" t="s">
         <v>34</v>
       </c>
@@ -24749,7 +24748,7 @@
         <v>54.948</v>
       </c>
     </row>
-    <row r="119" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A119" s="25" t="s">
         <v>52</v>
       </c>
@@ -24785,7 +24784,7 @@
         <v>54.533000000000001</v>
       </c>
     </row>
-    <row r="120" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A120" s="25" t="s">
         <v>52</v>
       </c>
@@ -24821,7 +24820,7 @@
         <v>54.533000000000001</v>
       </c>
     </row>
-    <row r="121" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A121" s="25" t="s">
         <v>52</v>
       </c>
@@ -24857,7 +24856,7 @@
         <v>54.533000000000001</v>
       </c>
     </row>
-    <row r="122" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A122" s="23" t="s">
         <v>47</v>
       </c>
@@ -24893,7 +24892,7 @@
         <v>53.738999999999997</v>
       </c>
     </row>
-    <row r="123" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A123" s="23" t="s">
         <v>47</v>
       </c>
@@ -24929,7 +24928,7 @@
         <v>53.738999999999997</v>
       </c>
     </row>
-    <row r="124" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A124" s="23" t="s">
         <v>47</v>
       </c>
@@ -25073,7 +25072,7 @@
         <v>54.98</v>
       </c>
     </row>
-    <row r="128" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A128" s="23" t="s">
         <v>56</v>
       </c>
@@ -25109,7 +25108,7 @@
         <v>52.53</v>
       </c>
     </row>
-    <row r="129" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A129" s="23" t="s">
         <v>56</v>
       </c>
@@ -25145,7 +25144,7 @@
         <v>52.53</v>
       </c>
     </row>
-    <row r="130" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A130" s="23" t="s">
         <v>56</v>
       </c>
@@ -25181,7 +25180,7 @@
         <v>52.53</v>
       </c>
     </row>
-    <row r="131" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A131" s="25" t="s">
         <v>39</v>
       </c>
@@ -25217,7 +25216,7 @@
         <v>52.033999999999999</v>
       </c>
     </row>
-    <row r="132" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A132" s="25" t="s">
         <v>39</v>
       </c>
@@ -25253,7 +25252,7 @@
         <v>52.033999999999999</v>
       </c>
     </row>
-    <row r="133" spans="1:12" hidden="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A133" s="25" t="s">
         <v>39</v>
       </c>
@@ -25290,13 +25289,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L133" xr:uid="{00000000-0009-0000-0000-000006000000}">
-    <filterColumn colId="3">
-      <filters>
-        <filter val="WCH"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:L133" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
   <conditionalFormatting sqref="G101:G133">
     <cfRule type="expression" dxfId="2" priority="1">
       <formula>$E101="R1"</formula>
@@ -27423,7 +27416,7 @@
         <v>43162</v>
       </c>
       <c r="D37" s="11" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E37" s="11" t="s">
         <v>223</v>
@@ -27636,7 +27629,6 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:R133"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -27703,7 +27695,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="2" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
         <v>25</v>
       </c>
@@ -27759,7 +27751,7 @@
         <v>55.215000000000003</v>
       </c>
     </row>
-    <row r="3" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A3" s="9" t="s">
         <v>25</v>
       </c>
@@ -27815,7 +27807,7 @@
         <v>55.215000000000003</v>
       </c>
     </row>
-    <row r="4" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
         <v>25</v>
       </c>
@@ -27871,7 +27863,7 @@
         <v>55.215000000000003</v>
       </c>
     </row>
-    <row r="5" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A5" s="11" t="s">
         <v>27</v>
       </c>
@@ -27927,7 +27919,7 @@
         <v>58.442</v>
       </c>
     </row>
-    <row r="6" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A6" s="11" t="s">
         <v>27</v>
       </c>
@@ -27983,7 +27975,7 @@
         <v>58.442</v>
       </c>
     </row>
-    <row r="7" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" s="11" t="s">
         <v>27</v>
       </c>
@@ -28207,7 +28199,7 @@
         <v>56.356000000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A11" s="11" t="s">
         <v>30</v>
       </c>
@@ -28263,7 +28255,7 @@
         <v>56.284999999999997</v>
       </c>
     </row>
-    <row r="12" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A12" s="11" t="s">
         <v>30</v>
       </c>
@@ -28319,7 +28311,7 @@
         <v>56.284999999999997</v>
       </c>
     </row>
-    <row r="13" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A13" s="11" t="s">
         <v>30</v>
       </c>
@@ -28543,7 +28535,7 @@
         <v>54.710999999999999</v>
       </c>
     </row>
-    <row r="17" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A17" s="11" t="s">
         <v>32</v>
       </c>
@@ -28599,7 +28591,7 @@
         <v>55.728000000000002</v>
       </c>
     </row>
-    <row r="18" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A18" s="11" t="s">
         <v>32</v>
       </c>
@@ -28655,7 +28647,7 @@
         <v>55.728000000000002</v>
       </c>
     </row>
-    <row r="19" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A19" s="11" t="s">
         <v>32</v>
       </c>
@@ -28711,7 +28703,7 @@
         <v>55.728000000000002</v>
       </c>
     </row>
-    <row r="20" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A20" s="9" t="s">
         <v>34</v>
       </c>
@@ -28767,7 +28759,7 @@
         <v>54.579000000000001</v>
       </c>
     </row>
-    <row r="21" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A21" s="9" t="s">
         <v>34</v>
       </c>
@@ -28823,7 +28815,7 @@
         <v>54.579000000000001</v>
       </c>
     </row>
-    <row r="22" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A22" s="9" t="s">
         <v>34</v>
       </c>
@@ -28879,7 +28871,7 @@
         <v>54.579000000000001</v>
       </c>
     </row>
-    <row r="23" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A23" s="11" t="s">
         <v>27</v>
       </c>
@@ -28935,7 +28927,7 @@
         <v>54.579000000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A24" s="11" t="s">
         <v>27</v>
       </c>
@@ -28991,7 +28983,7 @@
         <v>54.579000000000001</v>
       </c>
     </row>
-    <row r="25" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A25" s="11" t="s">
         <v>27</v>
       </c>
@@ -29047,7 +29039,7 @@
         <v>54.579000000000001</v>
       </c>
     </row>
-    <row r="26" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A26" s="9" t="s">
         <v>35</v>
       </c>
@@ -29103,7 +29095,7 @@
         <v>51.195</v>
       </c>
     </row>
-    <row r="27" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A27" s="9" t="s">
         <v>35</v>
       </c>
@@ -29159,7 +29151,7 @@
         <v>51.195</v>
       </c>
     </row>
-    <row r="28" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A28" s="9" t="s">
         <v>35</v>
       </c>
@@ -29383,7 +29375,7 @@
         <v>57.765999999999998</v>
       </c>
     </row>
-    <row r="32" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A32" s="9" t="s">
         <v>34</v>
       </c>
@@ -29439,7 +29431,7 @@
         <v>55.283000000000001</v>
       </c>
     </row>
-    <row r="33" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A33" s="9" t="s">
         <v>34</v>
       </c>
@@ -29495,7 +29487,7 @@
         <v>55.283000000000001</v>
       </c>
     </row>
-    <row r="34" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A34" s="9" t="s">
         <v>34</v>
       </c>
@@ -29551,7 +29543,7 @@
         <v>55.283000000000001</v>
       </c>
     </row>
-    <row r="35" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A35" s="11" t="s">
         <v>37</v>
       </c>
@@ -29607,7 +29599,7 @@
         <v>54.25</v>
       </c>
     </row>
-    <row r="36" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A36" s="11" t="s">
         <v>37</v>
       </c>
@@ -29663,7 +29655,7 @@
         <v>54.25</v>
       </c>
     </row>
-    <row r="37" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A37" s="11" t="s">
         <v>37</v>
       </c>
@@ -29719,7 +29711,7 @@
         <v>54.25</v>
       </c>
     </row>
-    <row r="38" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A38" s="9" t="s">
         <v>38</v>
       </c>
@@ -29775,7 +29767,7 @@
         <v>53.411999999999999</v>
       </c>
     </row>
-    <row r="39" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A39" s="9" t="s">
         <v>38</v>
       </c>
@@ -29831,7 +29823,7 @@
         <v>53.411999999999999</v>
       </c>
     </row>
-    <row r="40" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A40" s="9" t="s">
         <v>38</v>
       </c>
@@ -30049,7 +30041,7 @@
       </c>
       <c r="R43" s="11"/>
     </row>
-    <row r="44" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A44" s="9" t="s">
         <v>39</v>
       </c>
@@ -30105,7 +30097,7 @@
         <v>52.052999999999997</v>
       </c>
     </row>
-    <row r="45" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A45" s="9" t="s">
         <v>39</v>
       </c>
@@ -30161,7 +30153,7 @@
         <v>52.052999999999997</v>
       </c>
     </row>
-    <row r="46" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A46" s="9" t="s">
         <v>39</v>
       </c>
@@ -30217,7 +30209,7 @@
         <v>52.052999999999997</v>
       </c>
     </row>
-    <row r="47" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A47" s="11" t="s">
         <v>34</v>
       </c>
@@ -30273,7 +30265,7 @@
         <v>54.314999999999998</v>
       </c>
     </row>
-    <row r="48" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A48" s="11" t="s">
         <v>34</v>
       </c>
@@ -30329,7 +30321,7 @@
         <v>54.314999999999998</v>
       </c>
     </row>
-    <row r="49" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A49" s="11" t="s">
         <v>34</v>
       </c>
@@ -30385,7 +30377,7 @@
         <v>54.314999999999998</v>
       </c>
     </row>
-    <row r="50" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A50" s="9" t="s">
         <v>36</v>
       </c>
@@ -30441,7 +30433,7 @@
         <v>54.281999999999996</v>
       </c>
     </row>
-    <row r="51" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A51" s="9" t="s">
         <v>36</v>
       </c>
@@ -30497,7 +30489,7 @@
         <v>54.281999999999996</v>
       </c>
     </row>
-    <row r="52" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A52" s="9" t="s">
         <v>36</v>
       </c>
@@ -30721,7 +30713,7 @@
         <v>54.216999999999999</v>
       </c>
     </row>
-    <row r="56" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A56" s="9" t="s">
         <v>39</v>
       </c>
@@ -30777,7 +30769,7 @@
         <v>50.137999999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A57" s="9" t="s">
         <v>39</v>
       </c>
@@ -30833,7 +30825,7 @@
         <v>50.137999999999998</v>
       </c>
     </row>
-    <row r="58" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A58" s="9" t="s">
         <v>39</v>
       </c>
@@ -30889,7 +30881,7 @@
         <v>50.137999999999998</v>
       </c>
     </row>
-    <row r="59" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A59" s="11" t="s">
         <v>41</v>
       </c>
@@ -30945,7 +30937,7 @@
         <v>55.107999999999997</v>
       </c>
     </row>
-    <row r="60" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A60" s="11" t="s">
         <v>41</v>
       </c>
@@ -31001,7 +30993,7 @@
         <v>55.107999999999997</v>
       </c>
     </row>
-    <row r="61" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A61" s="11" t="s">
         <v>41</v>
       </c>
@@ -31057,7 +31049,7 @@
         <v>55.107999999999997</v>
       </c>
     </row>
-    <row r="62" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A62" s="9" t="s">
         <v>42</v>
       </c>
@@ -31113,7 +31105,7 @@
         <v>51.48</v>
       </c>
     </row>
-    <row r="63" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A63" s="9" t="s">
         <v>42</v>
       </c>
@@ -31169,7 +31161,7 @@
         <v>51.48</v>
       </c>
     </row>
-    <row r="64" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A64" s="9" t="s">
         <v>42</v>
       </c>
@@ -31393,7 +31385,7 @@
         <v>54.576000000000001</v>
       </c>
     </row>
-    <row r="68" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A68" s="9" t="s">
         <v>34</v>
       </c>
@@ -31449,7 +31441,7 @@
         <v>53.93</v>
       </c>
     </row>
-    <row r="69" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A69" s="9" t="s">
         <v>34</v>
       </c>
@@ -31505,7 +31497,7 @@
         <v>53.93</v>
       </c>
     </row>
-    <row r="70" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A70" s="9" t="s">
         <v>34</v>
       </c>
@@ -31561,7 +31553,7 @@
         <v>53.93</v>
       </c>
     </row>
-    <row r="71" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A71" s="11" t="s">
         <v>44</v>
       </c>
@@ -31617,7 +31609,7 @@
         <v>53.168999999999997</v>
       </c>
     </row>
-    <row r="72" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A72" s="11" t="s">
         <v>44</v>
       </c>
@@ -31673,7 +31665,7 @@
         <v>53.168999999999997</v>
       </c>
     </row>
-    <row r="73" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A73" s="11" t="s">
         <v>44</v>
       </c>
@@ -31729,7 +31721,7 @@
         <v>53.168999999999997</v>
       </c>
     </row>
-    <row r="74" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A74" s="9" t="s">
         <v>45</v>
       </c>
@@ -31785,7 +31777,7 @@
         <v>54.075000000000003</v>
       </c>
     </row>
-    <row r="75" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A75" s="9" t="s">
         <v>45</v>
       </c>
@@ -31841,7 +31833,7 @@
         <v>54.075000000000003</v>
       </c>
     </row>
-    <row r="76" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A76" s="9" t="s">
         <v>45</v>
       </c>
@@ -31897,7 +31889,7 @@
         <v>54.075000000000003</v>
       </c>
     </row>
-    <row r="77" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A77" s="11" t="s">
         <v>27</v>
       </c>
@@ -31953,7 +31945,7 @@
         <v>55.494999999999997</v>
       </c>
     </row>
-    <row r="78" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A78" s="11" t="s">
         <v>27</v>
       </c>
@@ -32009,7 +32001,7 @@
         <v>55.494999999999997</v>
       </c>
     </row>
-    <row r="79" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A79" s="11" t="s">
         <v>27</v>
       </c>
@@ -32065,7 +32057,7 @@
         <v>55.494999999999997</v>
       </c>
     </row>
-    <row r="80" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A80" s="9" t="s">
         <v>36</v>
       </c>
@@ -32121,7 +32113,7 @@
         <v>53.826000000000001</v>
       </c>
     </row>
-    <row r="81" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A81" s="9" t="s">
         <v>36</v>
       </c>
@@ -32177,7 +32169,7 @@
         <v>53.826000000000001</v>
       </c>
     </row>
-    <row r="82" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A82" s="9" t="s">
         <v>36</v>
       </c>
@@ -32233,7 +32225,7 @@
         <v>53.826000000000001</v>
       </c>
     </row>
-    <row r="83" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A83" s="11" t="s">
         <v>46</v>
       </c>
@@ -32289,7 +32281,7 @@
         <v>53.822000000000003</v>
       </c>
     </row>
-    <row r="84" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A84" s="11" t="s">
         <v>46</v>
       </c>
@@ -32345,7 +32337,7 @@
         <v>53.822000000000003</v>
       </c>
     </row>
-    <row r="85" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A85" s="11" t="s">
         <v>46</v>
       </c>
@@ -32569,7 +32561,7 @@
         <v>54.338000000000001</v>
       </c>
     </row>
-    <row r="89" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A89" s="11" t="s">
         <v>27</v>
       </c>
@@ -32625,7 +32617,7 @@
         <v>54.046999999999997</v>
       </c>
     </row>
-    <row r="90" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A90" s="11" t="s">
         <v>27</v>
       </c>
@@ -32681,7 +32673,7 @@
         <v>54.046999999999997</v>
       </c>
     </row>
-    <row r="91" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A91" s="11" t="s">
         <v>27</v>
       </c>
@@ -32737,7 +32729,7 @@
         <v>54.046999999999997</v>
       </c>
     </row>
-    <row r="92" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A92" s="9" t="s">
         <v>45</v>
       </c>
@@ -32793,7 +32785,7 @@
         <v>51.37</v>
       </c>
     </row>
-    <row r="93" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A93" s="9" t="s">
         <v>45</v>
       </c>
@@ -32849,7 +32841,7 @@
         <v>51.37</v>
       </c>
     </row>
-    <row r="94" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A94" s="9" t="s">
         <v>45</v>
       </c>
@@ -32905,7 +32897,7 @@
         <v>51.37</v>
       </c>
     </row>
-    <row r="95" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A95" s="11" t="s">
         <v>49</v>
       </c>
@@ -32961,7 +32953,7 @@
         <v>52.722999999999999</v>
       </c>
     </row>
-    <row r="96" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A96" s="11" t="s">
         <v>49</v>
       </c>
@@ -33017,7 +33009,7 @@
         <v>52.722999999999999</v>
       </c>
     </row>
-    <row r="97" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A97" s="11" t="s">
         <v>49</v>
       </c>
@@ -33073,7 +33065,7 @@
         <v>52.722999999999999</v>
       </c>
     </row>
-    <row r="98" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A98" s="9" t="s">
         <v>43</v>
       </c>
@@ -33129,7 +33121,7 @@
         <v>52.741999999999997</v>
       </c>
     </row>
-    <row r="99" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A99" s="9" t="s">
         <v>43</v>
       </c>
@@ -33185,7 +33177,7 @@
         <v>52.741999999999997</v>
       </c>
     </row>
-    <row r="100" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A100" s="9" t="s">
         <v>43</v>
       </c>
@@ -33241,7 +33233,7 @@
         <v>52.741999999999997</v>
       </c>
     </row>
-    <row r="101" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A101" s="11" t="s">
         <v>34</v>
       </c>
@@ -33295,7 +33287,7 @@
         <v>52.878999999999998</v>
       </c>
     </row>
-    <row r="102" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A102" s="11" t="s">
         <v>34</v>
       </c>
@@ -33349,7 +33341,7 @@
         <v>52.878999999999998</v>
       </c>
     </row>
-    <row r="103" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A103" s="11" t="s">
         <v>34</v>
       </c>
@@ -33403,7 +33395,7 @@
         <v>52.878999999999998</v>
       </c>
     </row>
-    <row r="104" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A104" s="9" t="s">
         <v>32</v>
       </c>
@@ -33457,7 +33449,7 @@
         <v>53.993000000000002</v>
       </c>
     </row>
-    <row r="105" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A105" s="9" t="s">
         <v>32</v>
       </c>
@@ -33511,7 +33503,7 @@
         <v>53.993000000000002</v>
       </c>
     </row>
-    <row r="106" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A106" s="9" t="s">
         <v>32</v>
       </c>
@@ -33565,7 +33557,7 @@
         <v>53.993000000000002</v>
       </c>
     </row>
-    <row r="107" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A107" s="11" t="s">
         <v>48</v>
       </c>
@@ -33576,7 +33568,7 @@
         <v>43162</v>
       </c>
       <c r="D107" s="11" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E107" s="11" t="s">
         <v>223</v>
@@ -33619,7 +33611,7 @@
         <v>54.491</v>
       </c>
     </row>
-    <row r="108" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A108" s="11" t="s">
         <v>48</v>
       </c>
@@ -33630,7 +33622,7 @@
         <v>43162</v>
       </c>
       <c r="D108" s="11" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E108" s="11" t="s">
         <v>191</v>
@@ -33673,7 +33665,7 @@
         <v>54.491</v>
       </c>
     </row>
-    <row r="109" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A109" s="11" t="s">
         <v>48</v>
       </c>
@@ -33684,7 +33676,7 @@
         <v>43162</v>
       </c>
       <c r="D109" s="11" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E109" s="11" t="s">
         <v>137</v>
@@ -33727,7 +33719,7 @@
         <v>54.491</v>
       </c>
     </row>
-    <row r="110" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A110" s="9" t="s">
         <v>46</v>
       </c>
@@ -33781,7 +33773,7 @@
         <v>51.802999999999997</v>
       </c>
     </row>
-    <row r="111" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A111" s="9" t="s">
         <v>46</v>
       </c>
@@ -33835,7 +33827,7 @@
         <v>51.802999999999997</v>
       </c>
     </row>
-    <row r="112" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A112" s="9" t="s">
         <v>46</v>
       </c>
@@ -33889,7 +33881,7 @@
         <v>51.802999999999997</v>
       </c>
     </row>
-    <row r="113" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A113" s="11" t="s">
         <v>28</v>
       </c>
@@ -33943,7 +33935,7 @@
         <v>51.274000000000001</v>
       </c>
     </row>
-    <row r="114" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A114" s="11" t="s">
         <v>28</v>
       </c>
@@ -33997,7 +33989,7 @@
         <v>51.274000000000001</v>
       </c>
     </row>
-    <row r="115" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A115" s="11" t="s">
         <v>28</v>
       </c>
@@ -34051,7 +34043,7 @@
         <v>51.274000000000001</v>
       </c>
     </row>
-    <row r="116" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A116" s="9" t="s">
         <v>34</v>
       </c>
@@ -34105,7 +34097,7 @@
         <v>52.695999999999998</v>
       </c>
     </row>
-    <row r="117" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A117" s="9" t="s">
         <v>34</v>
       </c>
@@ -34159,7 +34151,7 @@
         <v>52.695999999999998</v>
       </c>
     </row>
-    <row r="118" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A118" s="9" t="s">
         <v>34</v>
       </c>
@@ -34213,7 +34205,7 @@
         <v>52.695999999999998</v>
       </c>
     </row>
-    <row r="119" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A119" s="11" t="s">
         <v>52</v>
       </c>
@@ -34267,7 +34259,7 @@
         <v>54.171999999999997</v>
       </c>
     </row>
-    <row r="120" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A120" s="11" t="s">
         <v>52</v>
       </c>
@@ -34321,7 +34313,7 @@
         <v>54.171999999999997</v>
       </c>
     </row>
-    <row r="121" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A121" s="11" t="s">
         <v>52</v>
       </c>
@@ -34375,7 +34367,7 @@
         <v>54.171999999999997</v>
       </c>
     </row>
-    <row r="122" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A122" s="9" t="s">
         <v>47</v>
       </c>
@@ -34429,7 +34421,7 @@
         <v>52.085000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A123" s="9" t="s">
         <v>47</v>
       </c>
@@ -34483,7 +34475,7 @@
         <v>52.085000000000001</v>
       </c>
     </row>
-    <row r="124" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A124" s="9" t="s">
         <v>47</v>
       </c>
@@ -34699,7 +34691,7 @@
         <v>52.703000000000003</v>
       </c>
     </row>
-    <row r="128" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A128" s="9" t="s">
         <v>56</v>
       </c>
@@ -34753,7 +34745,7 @@
         <v>50.832999999999998</v>
       </c>
     </row>
-    <row r="129" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A129" s="9" t="s">
         <v>56</v>
       </c>
@@ -34807,7 +34799,7 @@
         <v>50.832999999999998</v>
       </c>
     </row>
-    <row r="130" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A130" s="9" t="s">
         <v>56</v>
       </c>
@@ -34861,7 +34853,7 @@
         <v>50.832999999999998</v>
       </c>
     </row>
-    <row r="131" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A131" s="11" t="s">
         <v>39</v>
       </c>
@@ -34915,7 +34907,7 @@
         <v>51.021999999999998</v>
       </c>
     </row>
-    <row r="132" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A132" s="11" t="s">
         <v>39</v>
       </c>
@@ -34969,7 +34961,7 @@
         <v>51.021999999999998</v>
       </c>
     </row>
-    <row r="133" spans="1:18" hidden="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A133" s="11" t="s">
         <v>39</v>
       </c>
@@ -35024,13 +35016,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R133" xr:uid="{00000000-0009-0000-0000-000008000000}">
-    <filterColumn colId="3">
-      <filters>
-        <filter val="WCH"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:R133" xr:uid="{00000000-0009-0000-0000-000008000000}"/>
   <conditionalFormatting sqref="I2:I133">
     <cfRule type="colorScale" priority="13">
       <colorScale>
@@ -35435,4 +35421,10 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{9d5ca952-e4a5-43e6-b17c-c01d313ad135}" enabled="0" method="" siteId="{9d5ca952-e4a5-43e6-b17c-c01d313ad135}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>